<commit_message>
Updated Changes for MWC & Acquisiton
</commit_message>
<xml_diff>
--- a/acquisition/Files/b2b_agentic_streamlit_demo_data.xlsx
+++ b/acquisition/Files/b2b_agentic_streamlit_demo_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sumandeep.a.kaur\Documents\B2B Agentic Screens Demo\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sumandeep.a.kaur\Documents\Demo-17Feb\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E501FF-423F-4668-936E-B16A0EEB73F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1878187A-9802-4BAE-8647-6BF0F78827D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="701" xr2:uid="{F9668476-116F-4EE7-B02C-E81D09556175}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Customer360" sheetId="10" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Customer360!$A$1:$Z$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Customer360!$A$1:$AV$10</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="320">
   <si>
     <t>unique_id</t>
   </si>
@@ -47,9 +47,6 @@
     <t>company_name</t>
   </si>
   <si>
-    <t>lead_priority_label</t>
-  </si>
-  <si>
     <t>20251017194732_1</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>Low</t>
-  </si>
-  <si>
     <t>20251017194732_6</t>
   </si>
   <si>
@@ -201,9 +195,6 @@
   </si>
   <si>
     <t>Headquarter Location</t>
-  </si>
-  <si>
-    <t>Funding Amount($)</t>
   </si>
   <si>
     <r>
@@ -371,9 +362,6 @@
     <t>2121 Rosecrans Avenue, Suite 6300, El Segundo, CA 90245 USA</t>
   </si>
   <si>
-    <t>163 M</t>
-  </si>
-  <si>
     <t>Acq &amp; Mergers | Awards &amp; Recognition</t>
   </si>
   <si>
@@ -1188,16 +1176,10 @@
     <t>A-Mark Precious Metals, now operating under the Gold.com brand, is a fully integrated alternative assets platform spanning precious metals trading, collectibles, auctions, and DTC marketplaces following the Monex acquisition.</t>
   </si>
   <si>
-    <t>$835M (Monex Acquisition – Jan 2026)</t>
-  </si>
-  <si>
     <t>Strong top-line growth with temporary margin compression driven by M&amp;A integration, rebranding, and platform expansion.</t>
   </si>
   <si>
     <t>Wolfspeed is a global leader in silicon carbide semiconductor technology supporting EVs, renewable energy, AI data centers, and advanced industrial systems.</t>
-  </si>
-  <si>
-    <t>$750M+ (CHIPS Act &amp; Strategic Financing)</t>
   </si>
   <si>
     <t>Revenue pressure and losses driven by restructuring and fab consolidation, offset by improved liquidity and long-term capacity investments.</t>
@@ -1500,12 +1482,739 @@
   <si>
     <t>Merchant Wholesalers, Durable Goods (NAICS: 423940)</t>
   </si>
+  <si>
+    <t>Company_Annual_ICT_Spending_Bucket</t>
+  </si>
+  <si>
+    <t>Company_Annual_HW_Spending_Bucket</t>
+  </si>
+  <si>
+    <t>Company_Annual_SW_Spending_Bucket</t>
+  </si>
+  <si>
+    <t>Company_Annual_Telco_Spending_Bucket</t>
+  </si>
+  <si>
+    <t>Company_Annual_IT_Services_Spending_Bucket</t>
+  </si>
+  <si>
+    <t>Spend_Potential_Tier</t>
+  </si>
+  <si>
+    <t>Spend_Summary</t>
+  </si>
+  <si>
+    <t>Intent_Domain_1</t>
+  </si>
+  <si>
+    <t>Score_1</t>
+  </si>
+  <si>
+    <t>Domain_1_Top_Keywords (Top 5)</t>
+  </si>
+  <si>
+    <t>Intent_Domain_2</t>
+  </si>
+  <si>
+    <t>Score_2</t>
+  </si>
+  <si>
+    <t>Domain_2_Top_Keywords (Top 5)</t>
+  </si>
+  <si>
+    <t>Intent_Domain_3</t>
+  </si>
+  <si>
+    <t>Score_3</t>
+  </si>
+  <si>
+    <t>Domain_3_Top_Keywords (Top 5)</t>
+  </si>
+  <si>
+    <t>Competitor_Products_Searched</t>
+  </si>
+  <si>
+    <t>Intent_Priority_Tier</t>
+  </si>
+  <si>
+    <t>Intent_Summary</t>
+  </si>
+  <si>
+    <t>Tech_Maturity_Tier</t>
+  </si>
+  <si>
+    <t>Tech_Maturity_Summary</t>
+  </si>
+  <si>
+    <t>Telco_Tech_Relevance</t>
+  </si>
+  <si>
+    <t>Telco_Tech_Relevance_Summary</t>
+  </si>
+  <si>
+    <t>Competitor_Tech_Present</t>
+  </si>
+  <si>
+    <t>$40M–$120M</t>
+  </si>
+  <si>
+    <t>$8M–$20M</t>
+  </si>
+  <si>
+    <t>$20M–$60M</t>
+  </si>
+  <si>
+    <t>$5M–$15M</t>
+  </si>
+  <si>
+    <t>$10M–$30M</t>
+  </si>
+  <si>
+    <t>Very High</t>
+  </si>
+  <si>
+    <t>$2M–$6M</t>
+  </si>
+  <si>
+    <t>$500K–$1.5M</t>
+  </si>
+  <si>
+    <t>$800K–$2M</t>
+  </si>
+  <si>
+    <t>$600K–$1.5M</t>
+  </si>
+  <si>
+    <t>$700K–$2M</t>
+  </si>
+  <si>
+    <t>$5M–$12M</t>
+  </si>
+  <si>
+    <t>$1M–$3M</t>
+  </si>
+  <si>
+    <t>$3M–$6M</t>
+  </si>
+  <si>
+    <t>$1M–$2.5M</t>
+  </si>
+  <si>
+    <t>$1.5M–$4M</t>
+  </si>
+  <si>
+    <t>$3M–$8M</t>
+  </si>
+  <si>
+    <t>$3M–$7M</t>
+  </si>
+  <si>
+    <t>$150M–$400M</t>
+  </si>
+  <si>
+    <t>$30M–$80M</t>
+  </si>
+  <si>
+    <t>$80M–$200M</t>
+  </si>
+  <si>
+    <t>$4M–$10M</t>
+  </si>
+  <si>
+    <t>$6M–$18M</t>
+  </si>
+  <si>
+    <t>$60M–$150M</t>
+  </si>
+  <si>
+    <t>$20M–$50M</t>
+  </si>
+  <si>
+    <t>$15M–$40M</t>
+  </si>
+  <si>
+    <t>Cisco, Fortinet, CrowdStrike, Okta</t>
+  </si>
+  <si>
+    <t>Teams integration, cloud file sharing, project collaboration tools, SaaS adoption, cloud backup</t>
+  </si>
+  <si>
+    <t>Microsoft, Cisco</t>
+  </si>
+  <si>
+    <t>Salesforce, AWS, Azure</t>
+  </si>
+  <si>
+    <t>SAP, Cisco</t>
+  </si>
+  <si>
+    <t>Cisco, SAP, CrowdStrike, Okta</t>
+  </si>
+  <si>
+    <t>AWS, Cloudflare, Microsoft</t>
+  </si>
+  <si>
+    <t>Cisco, Oracle Cloud, CrowdStrike</t>
+  </si>
+  <si>
+    <t>Strong signals around DNS security resilience, zero-trust reinforcement, and cloud infrastructure scaling. Likely evaluating security stack optimisation and redundancy upgrades to maintain global internet backbone reliability.</t>
+  </si>
+  <si>
+    <t>Post-acquisition integration may drive system consolidation and network standardisation across regional offices.</t>
+  </si>
+  <si>
+    <t>Retail expansion and product innovation signal growing need for resilient store connectivity, integrated CRM, and cloud scalability.</t>
+  </si>
+  <si>
+    <t>Privatization and acquisition may trigger ERP consolidation and plant-level infrastructure optimisation.</t>
+  </si>
+  <si>
+    <t>Portfolio restructuring and divestiture activity suggest technology rationalisation and cost-optimisation initiatives across global operations.</t>
+  </si>
+  <si>
+    <t>Post-M&amp;A platform consolidation and digital marketplace expansion signal sustained cloud and security investments.</t>
+  </si>
+  <si>
+    <t>Restructuring and liquidity recapitalisation likely driving infrastructure optimisation, cost efficiency programs, and security reinforcement.</t>
+  </si>
+  <si>
+    <t>Highly diversified, enterprise-grade global stack spanning cloud, security, IAM, networking, and DevOps. Mature governance and operational sophistication.</t>
+  </si>
+  <si>
+    <t>Critical reliance on low-latency, redundant backbone connectivity and DDoS protection creates opportunity in high-capacity Ethernet, secure edge services, and advanced DDoS mitigation.</t>
+  </si>
+  <si>
+    <t>Limited but functional cloud and SaaS adoption. Technology used operationally rather than strategically.</t>
+  </si>
+  <si>
+    <t>Multi-branch operations create opportunity for SD-WAN, secure site connectivity, and mobility bundle upgrades.</t>
+  </si>
+  <si>
+    <t>Modern cloud-first stack supporting retail growth and brand expansion.</t>
+  </si>
+  <si>
+    <t>Store rollout and omnichannel strategy increase demand for secure, scalable retail connectivity and SD-WAN.</t>
+  </si>
+  <si>
+    <t>Operationally mature but ERP-centric stack; likely evolving toward digital manufacturing transformation.</t>
+  </si>
+  <si>
+    <t>Industrial sites require resilient connectivity and segmented networks for production continuity.</t>
+  </si>
+  <si>
+    <t>Highly advanced, multi-layered enterprise stack with AI, automation, and mature governance.</t>
+  </si>
+  <si>
+    <t>Global retail footprint drives high MPLS/SD-WAN demand, store connectivity, and secure cloud access requirements.</t>
+  </si>
+  <si>
+    <t>Cloud-centric with strong SaaS and security adoption; scaling through acquisitions.</t>
+  </si>
+  <si>
+    <t>High-value online transactions increase dependency on secure, low-latency internet and CDN optimization.</t>
+  </si>
+  <si>
+    <t>Advanced semiconductor-grade tech stack integrating cloud, ERP, AI, and security systems.</t>
+  </si>
+  <si>
+    <t>Manufacturing fabs and R&amp;D hubs require ultra-reliable, high-bandwidth connectivity and segmented industrial networks.</t>
+  </si>
+  <si>
+    <t>Cisco, Fortinet, Symantec</t>
+  </si>
+  <si>
+    <t>AWS, Azure, Salesforce</t>
+  </si>
+  <si>
+    <t>Salesforce</t>
+  </si>
+  <si>
+    <t>Cisco, SAP, Okta, CrowdStrike</t>
+  </si>
+  <si>
+    <t>AWS, Cloudflare</t>
+  </si>
+  <si>
+    <t>Cisco, Oracle, Symantec</t>
+  </si>
+  <si>
+    <t>Mission-critical DNS operator with global backbone and security-heavy infrastructure requirements.</t>
+  </si>
+  <si>
+    <t>Regional fire protection firm with moderate branch connectivity and compliance needs.</t>
+  </si>
+  <si>
+    <t>Retail growth brand scaling cloud, CRM and store connectivity footprint.</t>
+  </si>
+  <si>
+    <t>Manufacturing enterprise requiring plant networking and ERP-integrated infrastructure.</t>
+  </si>
+  <si>
+    <t>Global retail conglomerate with large-scale cloud, ERP and AI investments.</t>
+  </si>
+  <si>
+    <t>Acquisition-led digital marketplace expanding secure cloud and integration stack.</t>
+  </si>
+  <si>
+    <t>Semiconductor manufacturer with fab-grade connectivity and hybrid cloud dependency.</t>
+  </si>
+  <si>
+    <t>Digital Infrastructure</t>
+  </si>
+  <si>
+    <t>Networking</t>
+  </si>
+  <si>
+    <t>Cloud &amp; Data</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>telecommunications backbone, DNS infrastructure, carrier diversity, high-availability networks, network resilience</t>
+  </si>
+  <si>
+    <t>DDoS mitigation, zero trust security, secure DNS, threat monitoring, perimeter defence</t>
+  </si>
+  <si>
+    <t>multi-cloud optimisation, hybrid cloud networking, data centre interconnect, latency optimisation, workload security</t>
+  </si>
+  <si>
+    <t>branch connectivity, SD-WAN optimisation, secure remote access, site networking, bandwidth reliability</t>
+  </si>
+  <si>
+    <t>firewall upgrades, endpoint security, compliance monitoring, secure access, data protection</t>
+  </si>
+  <si>
+    <t>retail cloud scaling, CRM optimisation, SaaS integration, customer analytics, POS connectivity</t>
+  </si>
+  <si>
+    <t>store connectivity, SD-WAN deployment, bandwidth expansion, retail resilience, latency optimisation</t>
+  </si>
+  <si>
+    <t>payment security, endpoint protection, secure access, compliance controls, firewall upgrades</t>
+  </si>
+  <si>
+    <t>factory networking, industrial connectivity, data centre interconnect, high-performance networking, redundancy</t>
+  </si>
+  <si>
+    <t>ERP integration, SaaS migration, analytics integration, workload optimisation, CRM modernisation</t>
+  </si>
+  <si>
+    <t>OT security, network segmentation, endpoint protection, compliance monitoring, secure access</t>
+  </si>
+  <si>
+    <t>global networking, cloud connectivity, data centre interconnect, carrier diversity, enterprise backbone</t>
+  </si>
+  <si>
+    <t>zero trust architecture, endpoint protection, identity governance, cloud security posture, threat monitoring</t>
+  </si>
+  <si>
+    <t>multi-cloud optimisation, AI analytics, ERP transformation, retail cloud scaling, workflow automation</t>
+  </si>
+  <si>
+    <t>e-commerce scaling, digital marketplace optimisation, API integration, workload performance, cloud resilience</t>
+  </si>
+  <si>
+    <t>CDN security, DDoS protection, financial compliance controls, secure transactions, threat monitoring</t>
+  </si>
+  <si>
+    <t>internet resilience, bandwidth scaling, secure connectivity, SD-WAN optimisation, latency reduction</t>
+  </si>
+  <si>
+    <t>data centre interconnect, fab connectivity, high-performance networking, carrier diversity, global backbone</t>
+  </si>
+  <si>
+    <t>hybrid cloud deployment, AI workloads, latency optimisation, data transfer efficiency, cloud scalability</t>
+  </si>
+  <si>
+    <t>zero trust framework, endpoint security, network segmentation, threat detection, secure access</t>
+  </si>
+  <si>
+    <t>AvePoint</t>
+  </si>
+  <si>
+    <t>d91f1f57-41e3-58d8-b46b-99a5ebb084b8</t>
+  </si>
+  <si>
+    <t>Advanced Integration Technology</t>
+  </si>
+  <si>
+    <t>https://www.aint.com/</t>
+  </si>
+  <si>
+    <t>AIT designs, manufactures and installs automated tooling and equipment for the assembly of aerospace structures, as well as friction stir weld equipment for diversified industrial markets.</t>
+  </si>
+  <si>
+    <t>https://www.avepoint.com/</t>
+  </si>
+  <si>
+    <t>+1 972 423 8354</t>
+  </si>
+  <si>
+    <t>+1 201 793 1111</t>
+  </si>
+  <si>
+    <t>150 - 300</t>
+  </si>
+  <si>
+    <t>$10M - $100M</t>
+  </si>
+  <si>
+    <t>$100M - $500M</t>
+  </si>
+  <si>
+    <t>AvePoint provides a unified data protection platform for enterprises, focusing on security, governance, and resilience in the AI-driven workplace. They help organizations manage their data across the full digital lifecycle.</t>
+  </si>
+  <si>
+    <t>Manufacturing</t>
+  </si>
+  <si>
+    <t>Information Technology</t>
+  </si>
+  <si>
+    <t>2805 E. Plano Pkwy, Suite 300, Plano, TX 75074 USA</t>
+  </si>
+  <si>
+    <t>525 Washington Blvd, Suite 1400 Jersey City, NJ 07310</t>
+  </si>
+  <si>
+    <t>• Cloud: AWS Amazon Web Services, Azure DNS, Amazon Web Hosting • Networking: Cisco Routers, Cisco Switches, Cisco Meraki, Cisco VPN, Cisco Wireless • Security: Cisco Firepower, Cisco Adaptive Security Appliance ASA, Sophos, Entrust, Firewall Software • Identity &amp; Access: AD360, Authentication Platforms • ERP: IFS ERP, SAP, Oracle, Microsoft SQL Server • Industrial &amp; CAD: Autodesk, CATIA V5, Siemens SIMATIC S7, Solidworks, Mastercam, FactoryTalk • Virtualization: VMware • Collaboration &amp; Productivity: Microsoft Office 365, Microsoft Exchange Online, Polycom • Hosting &amp; DNS: GoDaddy DNS, Apache Servers</t>
+  </si>
+  <si>
+    <t>Advanced industrial and engineering-centric stack integrating ERP, CAD/CAM, industrial automation, and enterprise networking infrastructure.</t>
+  </si>
+  <si>
+    <t>Industrial automation and plant systems require resilient, segmented, and high-bandwidth connectivity. Strong opportunity in secure WAN, SD-WAN, and carrier redundancy solutions.</t>
+  </si>
+  <si>
+    <t>• Cloud: AWS Amazon Web Services, Microsoft Azure, Google Cloud Platform, Amazon CloudFront, Amazon Route 53 • Networking &amp; CDN: CloudFlare, Rackspace, Verizon Wireless • Security: Microsoft 365 Defender, Microsoft Azure Sentinel, Sophos, Tenable Nessus, SentinelOne, Barracuda Email Security • Identity &amp; Access: Microsoft Active Directory, Microsoft Entra, OAuth, OpenSSL • CRM &amp; Marketing: Salesforce CRM, HubSpot, Marketo, LinkedIn Sales Navigator, Google Ads, Facebook Pixel • Data &amp; Analytics: Google Analytics, Tableau, Power BI, MongoDB, MySQL, Elasticsearch • DevOps &amp; Development: Docker, Kubernetes (K8s), HashiCorp Terraform, Git, Ansible, React, Angular, Node.js • Collaboration: Microsoft Teams, SharePoint Online, Outlook.com</t>
+  </si>
+  <si>
+    <t>Highly advanced digital-first enterprise stack combining multi-cloud, marketing automation, CRM, DevOps, analytics, and enterprise security platforms.</t>
+  </si>
+  <si>
+    <t>Heavy dependency on cloud delivery, CDN performance, and secure remote workforce access. Significant demand for high-capacity internet, SD-WAN, and secure edge connectivity.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Operating across </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>10 key cities</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> globally-
+• Plano, Texas 
+• Richmond, VA
+• Chesterfield Twp, Michigan
+• Bothell, Washington
+• Leganés, Spain
+• France
+• Germany
+• San Antonio, Texas
+• Grand Prairie, Texas
+• Canada</t>
+    </r>
+  </si>
+  <si>
+    <t>Industrial automation, ERP, CAD/CAM, and plant networking environments drive high hardware, software, and carrier-grade connectivity investment.</t>
+  </si>
+  <si>
+    <t>Multi-cloud, marketing automation, DevOps, analytics, and enterprise security platforms create very large-scale software, services, and high-capacity connectivity demand.</t>
+  </si>
+  <si>
+    <t>industrial networking, plant connectivity, data centre interconnect, carrier diversity, high-availability networks</t>
+  </si>
+  <si>
+    <t>multi-cloud optimisation, cloud scalability, CDN performance, workload distribution, data transfer efficiency</t>
+  </si>
+  <si>
+    <t>OT security, network segmentation, firewall upgrades, secure remote access, threat monitoring</t>
+  </si>
+  <si>
+    <t>zero trust architecture, SIEM platforms, endpoint detection, cloud security posture, threat analytics</t>
+  </si>
+  <si>
+    <t>ERP modernisation, hybrid cloud deployment, workload optimisation, analytics platforms, virtualisation</t>
+  </si>
+  <si>
+    <t>SD-WAN optimisation, global backbone connectivity, carrier benchmarking, network resilience, secure edge</t>
+  </si>
+  <si>
+    <t>Cisco, SAP, VMware</t>
+  </si>
+  <si>
+    <t>AWS, Microsoft Azure, Cloudflare, Salesforce</t>
+  </si>
+  <si>
+    <t>Active research around industrial connectivity resilience, OT security, and hybrid infrastructure modernisation initiatives.</t>
+  </si>
+  <si>
+    <t>Sustained enterprise-wide research into multi-cloud optimisation, advanced security architecture, and global connectivity benchmarking.</t>
+  </si>
+  <si>
+    <t>Cisco, SAP, Oracle, VMware, AWS, Azure</t>
+  </si>
+  <si>
+    <t>AWS, Azure, Salesforce, Cloudflare, Microsoft, SAP</t>
+  </si>
+  <si>
+    <t>Acq &amp; Mergers | Partnership &amp; Alliances | Business Expansion | New Product or Technology Launches | Fundings &amp; Capital Raises | Revenue &amp; Earnings | Customer/Market Focus | Future Guidance &amp; Strategic Outlook</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/AvePointInc</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/company/advanced-integration-technology/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/advancedintegrationtechnology/</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/company/avepoint</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/avepoint/</t>
+  </si>
+  <si>
+    <t>+24% (2025 vs 2024)</t>
+  </si>
+  <si>
+    <t>+348% (2025 vs 2024)</t>
+  </si>
+  <si>
+    <t>Strong ARR and revenue growth driven by accelerating SaaS expansion and operating leverage, supported by margin improvement and a strengthened cash position.</t>
+  </si>
+  <si>
+    <t>-0.9% (2025 vs 2024)</t>
+  </si>
+  <si>
+    <t>-66.7% (2025 vs 2024)</t>
+  </si>
+  <si>
+    <t>https://www.quiverquant.com/news/AvePoint+Announces+Acquisition+of+Ydentic+to+Enhance+MSP+Platform+and+Automation+Solutions, 
+https://www.cnbc.com/video/2025/09/19/avepoint-ceo-on-strategic-sgx-listing-and-accelerating-ai-integration.html,
+https://www.avepoint.com/news/avepoint-expands-channel-strategy-with-new-azure-data-protection-global-iamcp-partnership-and-enhanced-marketplace-integrations, 
+https://www.avepoint.com/news/avepoint-launches-new-avepoint-agentpulse-command-center-to-bring-security-controls-to-ai-agents,
+https://www.stocktitan.net/news/AVPT/ave-point-announces-pricing-of-public-5kw33b1w30zh.html,
+https://finance.yahoo.com/news/avepoint-reports-third-quarter-2025-financial-results.html,
+https://finance.yahoo.com/news/avepoint-report-finds-ai-rollouts-130000357.html,
+https://www.globenewswire.com/news-release/2025/09/19/3152933/0/en/AvePoint-Announces-Dual-Listing-on-the-Singapore-Exchange-to-Continue-Global-Expansion.html</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Acq &amp; Mergers:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AvePoint acquired Ydentic to strengthen its MSP automation and platform capabilities.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Business Expansion: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">AvePoint dual-listed on Nasdaq and SGX to accelerate global growth and market expansion.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Partnership &amp; Alliances:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AvePoint expanded its global channel ecosystem through a strategic IAMCP partnership for Azure Data Protection.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>New Product or Technology Launches:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AvePoint launched AgentPulse and expanded AI-driven data protection across its Confidence and Elements platforms.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fundings &amp; Capital Raises:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AvePoint priced a public offering of 7.37M shares to support strategic growth initiatives.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Revenue &amp; Earnings:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AvePoint delivered strong Q3 2025 results with 24% revenue growth, 38% SaaS growth, and ARR reaching $390M.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Customer/Market Focus:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AvePoint is advancing a multi-cloud strategy while expanding enterprise and MSP-led growth.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Future Guidance &amp; Strategic Outlook:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AvePoint projects continued growth in Q4 and FY2025, targeting $1B ARR by 2029.</t>
+    </r>
+  </si>
+  <si>
+    <t>ACC001</t>
+  </si>
+  <si>
+    <t>Security Network</t>
+  </si>
+  <si>
+    <t>Cloud Services</t>
+  </si>
+  <si>
+    <t>US Sites: • Jersey City, NJ (HQ) • Chicago, IL • Richmond, VA • Arlington, VA • Toronto, Canada | EMEA: • London, UK • Johannesburg, SA • Stockholm, Sweden • The Hague, Netherlands | APAC: • Melbourne, Australia • Sydney, Australia • Beijing, China • Changchun, China • Dalian, China</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1536,8 +2245,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1546,24 +2263,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.89999084444715716"/>
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1571,80 +2282,85 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1974,692 +2690,1512 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{308A49E9-B7EE-4B49-A4E8-64E2E285BF73}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:Z8"/>
+  <dimension ref="A1:AV10"/>
   <sheetFormatPr defaultColWidth="23" defaultRowHeight="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="24.7109375" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" style="13" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" customWidth="1"/>
-    <col min="7" max="7" width="24.7109375" style="13" customWidth="1"/>
-    <col min="8" max="8" width="24.7109375" customWidth="1"/>
-    <col min="9" max="9" width="45" customWidth="1"/>
-    <col min="10" max="10" width="24.7109375" customWidth="1"/>
-    <col min="11" max="11" width="24.7109375" style="16" customWidth="1"/>
-    <col min="12" max="14" width="24.7109375" customWidth="1"/>
-    <col min="15" max="15" width="49.5703125" customWidth="1"/>
-    <col min="16" max="16" width="33.7109375" customWidth="1"/>
-    <col min="17" max="19" width="24.7109375" customWidth="1"/>
-    <col min="20" max="20" width="94.5703125" customWidth="1"/>
-    <col min="21" max="21" width="122.42578125" customWidth="1"/>
-    <col min="22" max="24" width="54.28515625" customWidth="1"/>
-    <col min="25" max="25" width="24.7109375" customWidth="1"/>
+    <col min="1" max="4" width="22.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" style="5" customWidth="1"/>
+    <col min="8" max="9" width="22.7109375" style="2" customWidth="1"/>
+    <col min="10" max="16" width="22.7109375" style="1" customWidth="1"/>
+    <col min="17" max="25" width="22.7109375" style="3" customWidth="1"/>
+    <col min="26" max="26" width="22.7109375" style="4" customWidth="1"/>
+    <col min="27" max="28" width="22.7109375" style="3" customWidth="1"/>
+    <col min="29" max="29" width="22.7109375" style="4" customWidth="1"/>
+    <col min="30" max="31" width="22.7109375" style="3" customWidth="1"/>
+    <col min="32" max="32" width="22.7109375" style="4" customWidth="1"/>
+    <col min="33" max="34" width="22.7109375" style="3" customWidth="1"/>
+    <col min="35" max="35" width="22.7109375" style="4" customWidth="1"/>
+    <col min="36" max="43" width="22.7109375" style="2" customWidth="1"/>
+    <col min="44" max="44" width="22.7109375" style="1" customWidth="1"/>
+    <col min="45" max="48" width="22.7109375" style="2" customWidth="1"/>
+    <col min="49" max="16384" width="23" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:48" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="K1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="S1" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="T1" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="V1" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="Y1" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="Z1" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="AA1" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="AB1" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="AC1" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="AD1" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="AE1" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="AF1" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="AG1" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="AH1" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="AI1" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="AJ1" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="AK1" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL1" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AM1" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AN1" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="AO1" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="AP1" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="AQ1" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="AR1" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="AS1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="AT1" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="AU1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="AV1" s="6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:48" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="7">
+        <v>1995</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="N2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="O2" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q2" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="R2" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="S2" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="T2" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="U2" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="V2" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="W2" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="X2" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="Y2" s="7">
+        <v>93</v>
+      </c>
+      <c r="Z2" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="AA2" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="AB2" s="7">
+        <v>89</v>
+      </c>
+      <c r="AC2" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="AD2" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="AE2" s="7">
+        <v>84</v>
+      </c>
+      <c r="AF2" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="AG2" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="AH2" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI2" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="AJ2" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="AK2" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="AL2" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AM2" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="AN2" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="AO2" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AP2" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AQ2" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR2" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="AS2" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="AT2" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="AU2" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="AV2" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:48" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" s="7">
+        <v>1998</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="J3" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="K3" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="T3" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="U3" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="V3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="W3" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="X3" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="Y3" s="7">
+        <v>64</v>
+      </c>
+      <c r="Z3" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="AA3" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="AB3" s="7">
+        <v>58</v>
+      </c>
+      <c r="AC3" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="AD3" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="AE3" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="AF3" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG3" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="AH3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AI3" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="AJ3" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AK3" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AL3" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AM3" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AN3" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AO3" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AP3" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AQ3" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="AR3" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="L1" s="5" t="s">
+      <c r="AS3" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="AT3" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="AU3" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="AV3" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:48" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="7">
+        <v>2013</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="J4" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="M1" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="N1" t="s">
+      <c r="K4" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="R4" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="S4" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="T4" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="U4" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="V4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="W4" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="X4" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="Y4" s="7">
+        <v>78</v>
+      </c>
+      <c r="Z4" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="AA4" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="AB4" s="7">
+        <v>70</v>
+      </c>
+      <c r="AC4" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="AD4" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="AE4" s="7">
+        <v>63</v>
+      </c>
+      <c r="AF4" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG4" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="AH4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI4" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="AJ4" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AK4" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AL4" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AM4" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AN4" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AO4" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AP4" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="AQ4" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="AR4" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="AS4" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="AT4" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="AU4" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="AV4" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:48" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="7">
+        <v>1994</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="S5" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="T5" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="U5" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="V5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="W5" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="X5" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="Y5" s="7">
+        <v>82</v>
+      </c>
+      <c r="Z5" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="AA5" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="AB5" s="7">
+        <v>74</v>
+      </c>
+      <c r="AC5" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="AD5" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="AE5" s="7">
+        <v>69</v>
+      </c>
+      <c r="AF5" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="AG5" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="AH5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AI5" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="AJ5" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AK5" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AL5" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AM5" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AN5" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AO5" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AP5" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="AQ5" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="AR5" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS5" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="AT5" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU5" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="AV5" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:48" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E6" s="7">
+        <v>1899</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="S6" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="T6" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="U6" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="V6" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="W6" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="X6" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="Y6" s="7">
+        <v>91</v>
+      </c>
+      <c r="Z6" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="AA6" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="AB6" s="7">
+        <v>88</v>
+      </c>
+      <c r="AC6" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="AD6" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="AE6" s="7">
+        <v>85</v>
+      </c>
+      <c r="AF6" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="AG6" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="AH6" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI6" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="AJ6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AK6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AL6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AM6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AN6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AO6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="AP6" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="AQ6" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="AR6" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="AS6" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="AT6" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="AU6" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="AV6" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:48" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E7" s="7">
+        <v>1965</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T7" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="U7" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="V7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="Y7" s="7">
+        <v>83</v>
+      </c>
+      <c r="Z7" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="AA7" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="AB7" s="7">
+        <v>78</v>
+      </c>
+      <c r="AC7" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="AD7" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="AE7" s="7">
+        <v>72</v>
+      </c>
+      <c r="AF7" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="AG7" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="AH7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI7" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="AJ7" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="AK7" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="AL7" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="AM7" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="AN7" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="AO7" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="AP7" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="AQ7" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="AR7" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="AS7" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="AT7" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="AU7" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="AV7" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:48" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E8" s="7">
+        <v>2015</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K8" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="O1" t="s">
-        <v>83</v>
-      </c>
-      <c r="P1" t="s">
+      <c r="L8" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="S8" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="T8" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="U8" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="V8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="W8" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="X8" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="Y8" s="7">
+        <v>89</v>
+      </c>
+      <c r="Z8" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="AA8" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="AB8" s="7">
         <v>84</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="AC8" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="AD8" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="AE8" s="7">
+        <v>81</v>
+      </c>
+      <c r="AF8" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="AG8" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="AH8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI8" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="AJ8" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="AK8" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="AL8" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="AM8" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="AN8" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO8" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="AP8" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="AQ8" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="AR8" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="AS8" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="AT8" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="AU8" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV8" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:48" s="3" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="E9" s="12">
+        <v>2007</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="M9" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="N9" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="O9" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="P9" s="12" t="s">
+        <v>301</v>
+      </c>
+      <c r="Q9" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="R9" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="S9" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="T9" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="U9" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="V9" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="W9" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="X9" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="Y9" s="14">
+        <v>88</v>
+      </c>
+      <c r="Z9" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="AA9" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="AB9" s="14">
+        <v>84</v>
+      </c>
+      <c r="AC9" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="AD9" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="AE9" s="14">
+        <v>79</v>
+      </c>
+      <c r="AF9" s="14" t="s">
+        <v>295</v>
+      </c>
+      <c r="AG9" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="AH9" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI9" s="14" t="s">
+        <v>299</v>
+      </c>
+      <c r="AJ9" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AK9" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AL9" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AM9" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AN9" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AO9" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AP9" s="12"/>
+      <c r="AQ9" s="12"/>
+      <c r="AR9" s="14"/>
+      <c r="AS9" s="12"/>
+      <c r="AT9" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="AU9" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="AV9" s="12" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="10" spans="1:48" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="E10" s="12">
+        <v>2001</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="J10" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="L10" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="M10" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="N10" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="O10" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="P10" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q10" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="R10" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="S10" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="T10" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="U10" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="V10" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="W10" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="X10" s="14" t="s">
+        <v>317</v>
+      </c>
+      <c r="Y10" s="14">
         <v>85</v>
       </c>
-      <c r="R1" t="s">
-        <v>86</v>
-      </c>
-      <c r="S1" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="T1" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="U1" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="Z1" s="6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="E2" s="12">
-        <v>1995</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="K2" s="15" t="s">
+      <c r="Z10" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="AA10" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="AB10" s="14">
+        <v>80</v>
+      </c>
+      <c r="AC10" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="AD10" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="AE10" s="14">
         <v>78</v>
       </c>
-      <c r="L2" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="M2" t="s">
-        <v>95</v>
-      </c>
-      <c r="N2" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="O2" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="P2" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q2" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="R2" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="U2" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="V2" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="W2" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="Y2" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z2" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="E3" s="12">
-        <v>1998</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M3" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="N3" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="P3" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q3" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="R3" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="T3" s="2" t="s">
+      <c r="AF10" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="AG10" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="AH10" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI10" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="AJ10" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="AK10" s="15" t="s">
+        <v>309</v>
+      </c>
+      <c r="AL10" s="15" t="s">
+        <v>310</v>
+      </c>
+      <c r="AM10" s="15" t="s">
+        <v>312</v>
+      </c>
+      <c r="AN10" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="U3" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="V3" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="X3" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="Z3" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E4" s="12">
-        <v>2013</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="K4" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="O4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="P4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="R4" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="T4" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="U4" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V4" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="X4" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="Y4" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E5" s="12">
-        <v>1994</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="K5" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M5" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="N5" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="O5" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="P5" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q5" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="R5" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="T5" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="U5" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="V5" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="W5" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="X5" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="Y5" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z5" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="E6" s="12">
-        <v>1899</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M6" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="N6" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="O6" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="P6" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q6" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="R6" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="S6" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="U6" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="V6" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="W6" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="X6" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="Y6" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z6" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="E7" s="12">
-        <v>1965</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="K7" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="M7" t="s">
-        <v>144</v>
-      </c>
-      <c r="N7" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="P7" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q7" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="R7" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="U7" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="V7" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="W7" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="X7" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="Y7" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="Z7" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="E8" s="12">
-        <v>2015</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="K8" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="M8" t="s">
-        <v>147</v>
-      </c>
-      <c r="N8" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="O8" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="P8" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q8" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="R8" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="S8" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="U8" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="V8" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="W8" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="X8" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="Y8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z8" s="7" t="s">
-        <v>21</v>
+      <c r="AO10" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="AP10" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="AQ10" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="AR10" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="AS10" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="AT10" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="AU10" s="14" t="s">
+        <v>308</v>
+      </c>
+      <c r="AV10" s="12" t="s">
+        <v>273</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z8" xr:uid="{308A49E9-B7EE-4B49-A4E8-64E2E285BF73}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z8">
-      <sortCondition sortBy="cellColor" ref="B1:B8" dxfId="0"/>
-    </sortState>
+  <autoFilter ref="A1:AV10" xr:uid="{308A49E9-B7EE-4B49-A4E8-64E2E285BF73}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="ACC001"/>
+      </filters>
+    </filterColumn>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1" xr:uid="{3E169230-EEBD-4556-8C30-13114CFAF121}"/>
-    <hyperlink ref="W2" r:id="rId2" xr:uid="{9BA68AE6-B3C3-4303-8488-B5E7A5F37D17}"/>
-    <hyperlink ref="W8" r:id="rId3" xr:uid="{732B2BAC-568B-4A88-AED6-5437C7103AA3}"/>
-    <hyperlink ref="W6" r:id="rId4" xr:uid="{C19A1A07-C22F-4EEA-A6D8-6A5F25C63B0E}"/>
-    <hyperlink ref="X8" r:id="rId5" xr:uid="{7F268939-E672-4EEC-A363-66CC74CDE7B1}"/>
-    <hyperlink ref="X4" r:id="rId6" xr:uid="{FFEB7E23-22B9-4630-9E70-C558D8CD5DBB}"/>
-    <hyperlink ref="X3" r:id="rId7" xr:uid="{7C202E08-23A9-4042-951E-59FCDC3473E4}"/>
-    <hyperlink ref="V6" r:id="rId8" xr:uid="{75F07DC8-AA4D-42C9-B1C0-A7FC6CA9B398}"/>
-    <hyperlink ref="V4" r:id="rId9" xr:uid="{8CF0AE0F-BF23-4EE1-A07F-F270217E4FC8}"/>
-    <hyperlink ref="V3" r:id="rId10" xr:uid="{B5757B20-8B67-46B3-BC04-64C157E23CF8}"/>
-    <hyperlink ref="V2" r:id="rId11" xr:uid="{42E614CE-929E-48F5-B226-18F87BFAE512}"/>
+    <hyperlink ref="AR2" r:id="rId1" xr:uid="{3E169230-EEBD-4556-8C30-13114CFAF121}"/>
+    <hyperlink ref="AT2" r:id="rId2" xr:uid="{9BA68AE6-B3C3-4303-8488-B5E7A5F37D17}"/>
+    <hyperlink ref="AT8" r:id="rId3" xr:uid="{732B2BAC-568B-4A88-AED6-5437C7103AA3}"/>
+    <hyperlink ref="AT6" r:id="rId4" xr:uid="{C19A1A07-C22F-4EEA-A6D8-6A5F25C63B0E}"/>
+    <hyperlink ref="AU8" r:id="rId5" xr:uid="{7F268939-E672-4EEC-A363-66CC74CDE7B1}"/>
+    <hyperlink ref="AU4" r:id="rId6" xr:uid="{FFEB7E23-22B9-4630-9E70-C558D8CD5DBB}"/>
+    <hyperlink ref="AU3" r:id="rId7" xr:uid="{7C202E08-23A9-4042-951E-59FCDC3473E4}"/>
+    <hyperlink ref="AS6" r:id="rId8" xr:uid="{75F07DC8-AA4D-42C9-B1C0-A7FC6CA9B398}"/>
+    <hyperlink ref="AS4" r:id="rId9" xr:uid="{8CF0AE0F-BF23-4EE1-A07F-F270217E4FC8}"/>
+    <hyperlink ref="AS3" r:id="rId10" xr:uid="{B5757B20-8B67-46B3-BC04-64C157E23CF8}"/>
+    <hyperlink ref="AS2" r:id="rId11" xr:uid="{42E614CE-929E-48F5-B226-18F87BFAE512}"/>
     <hyperlink ref="C7" r:id="rId12" xr:uid="{000DCBBE-9B71-4A19-A589-0CED4B912D3E}"/>
+    <hyperlink ref="C9" r:id="rId13" xr:uid="{B9E512D9-BB2A-4A40-966D-C792685205AC}"/>
+    <hyperlink ref="C10" r:id="rId14" xr:uid="{48236C4B-E14C-4D4E-8D3B-B9DE74DE85A5}"/>
+    <hyperlink ref="AR10" r:id="rId15" display="https://www.quiverquant.com/news/AvePoint+Announces+Acquisition+of+Ydentic+to+Enhance+MSP+Platform+and+Automation+Solutions" xr:uid="{379D7CCD-8361-4D94-BB54-D0CE635E59A9}"/>
+    <hyperlink ref="AS10" r:id="rId16" xr:uid="{33C342B4-EC3B-42F9-96F3-42B9837C1CB3}"/>
+    <hyperlink ref="AU9" r:id="rId17" display="https://www.instagram.com/advancedintegrationtechnology/?utm_source=chatgpt.com" xr:uid="{D98A1331-0682-4BC8-B5ED-EA563457C41F}"/>
+    <hyperlink ref="AT10" r:id="rId18" display="https://www.linkedin.com/company/avepoint?utm_source=chatgpt.com" xr:uid="{9563144E-AEC7-47AE-AD0F-45E8FFAFD1B5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId13"/>
+  <pageSetup orientation="portrait" r:id="rId19"/>
 </worksheet>
 </file>
 

</xml_diff>